<commit_message>
feature: Ability item/unit 로직 추가 구현.
</commit_message>
<xml_diff>
--- a/input/Domains/Game/UnitTable.xlsx
+++ b/input/Domains/Game/UnitTable.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/maoshy/Documents/Projects/devian/input/Domains/Game/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3F2683B-C901-3347-AA8B-A1BF339E85C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E340A7D-3C2B-5040-8F2D-79974CB7556E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="44620" yWindow="-2060" windowWidth="25640" windowHeight="20800" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6240" yWindow="500" windowWidth="25640" windowHeight="20800" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UNIT_HERO" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="30">
   <si>
     <t>unitId</t>
   </si>
@@ -113,6 +113,14 @@
   </si>
   <si>
     <t>unit_monster_001</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>group:true</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>index</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -480,9 +488,6 @@
       <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
-        <v>3</v>
-      </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
@@ -496,9 +501,6 @@
       </c>
       <c r="D2" t="s">
         <v>4</v>
-      </c>
-      <c r="E2" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -568,115 +570,160 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45402A86-376A-5B4F-A1D8-495F727FDD37}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="13.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
         <v>19</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
         <v>19</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
         <v>18</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
         <v>18</v>
       </c>
-      <c r="B8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
+      <c r="C8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
         <v>18</v>
       </c>
-      <c r="B9">
+      <c r="C9">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
+    <row r="10" spans="1:4">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
         <v>18</v>
       </c>
-      <c r="B10">
+      <c r="C10">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
+    <row r="12" spans="1:4">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
         <v>18</v>
       </c>
-      <c r="B12">
+      <c r="C12">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
+    <row r="13" spans="1:4">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
         <v>18</v>
       </c>
-      <c r="B13">
+      <c r="C13">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
+    <row r="14" spans="1:4">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
         <v>18</v>
       </c>
-      <c r="B14">
+      <c r="C14">
         <v>10</v>
       </c>
     </row>
@@ -688,13 +735,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -704,11 +751,8 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4">
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -718,16 +762,13 @@
       <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -737,11 +778,8 @@
       <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -754,115 +792,160 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{288F280D-250F-B046-AFBF-D446BE65CBC1}">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17"/>
   <cols>
-    <col min="1" max="1" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
+        <v>29</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:2">
+      <c r="D2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
+      <c r="B3" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="B4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
+    <row r="5" spans="1:4">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" t="s">
         <v>27</v>
       </c>
-      <c r="B5">
+      <c r="C5">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
+    <row r="6" spans="1:4">
+      <c r="A6">
+        <v>2</v>
+      </c>
+      <c r="B6" t="s">
         <v>27</v>
       </c>
-      <c r="B6">
+      <c r="C6">
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
+    <row r="7" spans="1:4">
+      <c r="A7">
+        <v>3</v>
+      </c>
+      <c r="B7" t="s">
         <v>26</v>
       </c>
-      <c r="B7">
+      <c r="C7">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
-      <c r="A8" t="s">
+    <row r="8" spans="1:4">
+      <c r="A8">
+        <v>4</v>
+      </c>
+      <c r="B8" t="s">
         <v>26</v>
       </c>
-      <c r="B8">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
+      <c r="C8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9" t="s">
         <v>26</v>
       </c>
-      <c r="B9">
+      <c r="C9">
         <v>5</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
+    <row r="10" spans="1:4">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10" t="s">
         <v>26</v>
       </c>
-      <c r="B10">
+      <c r="C10">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
+    <row r="11" spans="1:4">
+      <c r="A11">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
         <v>26</v>
       </c>
-      <c r="B11">
+      <c r="C11">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
-      <c r="A12" t="s">
+    <row r="12" spans="1:4">
+      <c r="A12">
+        <v>8</v>
+      </c>
+      <c r="B12" t="s">
         <v>26</v>
       </c>
-      <c r="B12">
+      <c r="C12">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
-      <c r="A13" t="s">
+    <row r="13" spans="1:4">
+      <c r="A13">
+        <v>9</v>
+      </c>
+      <c r="B13" t="s">
         <v>26</v>
       </c>
-      <c r="B13">
+      <c r="C13">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
-      <c r="A14" t="s">
+    <row r="14" spans="1:4">
+      <c r="A14">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
         <v>26</v>
       </c>
-      <c r="B14">
+      <c r="C14">
         <v>10</v>
       </c>
     </row>

</xml_diff>